<commit_message>
Initial commit - ScootDR project
</commit_message>
<xml_diff>
--- a/Fleet Mileage.xlsx
+++ b/Fleet Mileage.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10913"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11028"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/DATA/Business/scootdr/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36098707-0478-8F45-854D-DCF218821680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E7DE1D3-73BD-CD41-B04B-DE9D9A383473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="25520" windowHeight="15500" xr2:uid="{DD62F603-65F5-B64B-908C-44E0CEED2B19}"/>
   </bookViews>
@@ -827,16 +827,18 @@
         <v>1</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C2" s="19">
-        <v>41904</v>
+        <v>51080</v>
       </c>
       <c r="D2" s="19">
-        <v>45000</v>
+        <v>54000</v>
       </c>
       <c r="E2" s="3"/>
-      <c r="F2" s="21"/>
+      <c r="F2" t="s">
+        <v>63</v>
+      </c>
       <c r="G2" s="6"/>
       <c r="H2" s="7" t="s">
         <v>6</v>
@@ -847,16 +849,18 @@
         <v>2</v>
       </c>
       <c r="B3" s="14" t="s">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="C3" s="19">
-        <v>44680</v>
+        <v>50950</v>
       </c>
       <c r="D3" s="19">
-        <v>48000</v>
+        <v>53000</v>
       </c>
       <c r="E3" s="3"/>
-      <c r="F3" s="21"/>
+      <c r="F3" t="s">
+        <v>63</v>
+      </c>
       <c r="G3" s="8"/>
       <c r="H3" s="9" t="s">
         <v>50</v>
@@ -867,17 +871,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="14" t="s">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="C4" s="19">
-        <v>51080</v>
+        <v>48003</v>
       </c>
       <c r="D4" s="19">
-        <v>54000</v>
-      </c>
-      <c r="E4" s="3"/>
-      <c r="F4" t="s">
-        <v>63</v>
+        <v>51000</v>
       </c>
       <c r="G4" s="10"/>
       <c r="H4" s="11" t="s">
@@ -889,14 +889,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C5" s="19">
-        <v>48003</v>
+        <v>44680</v>
       </c>
       <c r="D5" s="19">
-        <v>51000</v>
-      </c>
+        <v>48000</v>
+      </c>
+      <c r="E5" s="3"/>
+      <c r="F5" s="21"/>
       <c r="G5" s="13"/>
       <c r="H5" s="7" t="s">
         <v>9</v>
@@ -907,17 +909,17 @@
         <v>5</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C6" s="19">
-        <v>50950</v>
+        <v>41969</v>
       </c>
       <c r="D6" s="19">
-        <v>53000</v>
+        <v>45000</v>
       </c>
       <c r="E6" s="3"/>
-      <c r="F6" t="s">
-        <v>63</v>
+      <c r="F6" s="21" t="s">
+        <v>64</v>
       </c>
       <c r="G6" s="4"/>
       <c r="H6" s="4"/>
@@ -927,18 +929,16 @@
         <v>6</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="C7" s="19">
-        <v>41969</v>
+        <v>41904</v>
       </c>
       <c r="D7" s="19">
         <v>45000</v>
       </c>
       <c r="E7" s="3"/>
-      <c r="F7" s="21" t="s">
-        <v>64</v>
-      </c>
+      <c r="F7" s="21"/>
       <c r="G7" s="4"/>
       <c r="H7" s="4"/>
     </row>
@@ -946,13 +946,13 @@
       <c r="A8" s="2">
         <v>7</v>
       </c>
-      <c r="B8" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="C8" s="19">
-        <v>38901</v>
-      </c>
-      <c r="D8" s="19">
+      <c r="B8" s="18" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="18">
+        <v>39172</v>
+      </c>
+      <c r="D8" s="18">
         <v>42000</v>
       </c>
       <c r="E8" s="3"/>
@@ -964,17 +964,16 @@
       <c r="A9" s="2">
         <v>8</v>
       </c>
-      <c r="B9" s="20" t="s">
-        <v>18</v>
+      <c r="B9" s="18" t="s">
+        <v>20</v>
       </c>
       <c r="C9" s="18">
-        <v>36148</v>
+        <v>38988</v>
       </c>
       <c r="D9" s="18">
-        <v>39000</v>
-      </c>
-      <c r="E9" s="3"/>
-      <c r="F9" s="21"/>
+        <v>42000</v>
+      </c>
+      <c r="E9" s="12"/>
       <c r="G9" s="4"/>
       <c r="H9" s="4"/>
     </row>
@@ -983,10 +982,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>7</v>
+        <v>30</v>
       </c>
       <c r="C10" s="18">
-        <v>39172</v>
+        <v>38901</v>
       </c>
       <c r="D10" s="18">
         <v>42000</v>
@@ -1000,16 +999,17 @@
       <c r="A11" s="2">
         <v>10</v>
       </c>
-      <c r="B11" s="18" t="s">
-        <v>20</v>
+      <c r="B11" s="20" t="s">
+        <v>18</v>
       </c>
       <c r="C11" s="18">
-        <v>38988</v>
+        <v>36148</v>
       </c>
       <c r="D11" s="18">
-        <v>42000</v>
-      </c>
-      <c r="E11" s="12"/>
+        <v>39000</v>
+      </c>
+      <c r="E11" s="3"/>
+      <c r="F11" s="21"/>
       <c r="G11" s="4"/>
       <c r="H11" s="4"/>
     </row>
@@ -1018,42 +1018,43 @@
         <v>11</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>5</v>
+        <v>27</v>
       </c>
       <c r="C12" s="17">
-        <v>14866</v>
+        <v>33062</v>
       </c>
       <c r="D12" s="17">
-        <v>18000</v>
-      </c>
+        <v>36000</v>
+      </c>
+      <c r="E12" s="3"/>
+      <c r="F12" s="21"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="2">
         <v>12</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="C13" s="17">
-        <v>12047</v>
+        <v>33042</v>
       </c>
       <c r="D13" s="17">
-        <v>15000</v>
-      </c>
-      <c r="E13" s="3"/>
+        <v>36000</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="2">
         <v>13</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>10</v>
+        <v>29</v>
       </c>
       <c r="C14" s="17">
-        <v>14916</v>
+        <v>32993</v>
       </c>
       <c r="D14" s="17">
-        <v>18000</v>
+        <v>36000</v>
       </c>
       <c r="E14" s="3"/>
       <c r="F14" s="21"/>
@@ -1063,28 +1064,32 @@
         <v>14</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="C15" s="17">
-        <v>17822</v>
+        <v>32945</v>
       </c>
       <c r="D15" s="17">
-        <v>21000</v>
-      </c>
-      <c r="E15" s="3"/>
+        <v>36000</v>
+      </c>
+      <c r="E15" s="15"/>
+      <c r="F15" s="21"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A16" s="2">
         <v>15</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C16" s="17">
-        <v>21012</v>
+        <v>30014</v>
       </c>
       <c r="D16" s="17">
-        <v>24000</v>
+        <v>33000</v>
+      </c>
+      <c r="F16" s="21" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
@@ -1092,17 +1097,16 @@
         <v>16</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C17" s="17">
-        <v>30014</v>
+        <v>29918</v>
       </c>
       <c r="D17" s="17">
         <v>33000</v>
       </c>
-      <c r="F17" s="21" t="s">
-        <v>64</v>
-      </c>
+      <c r="E17" s="3"/>
+      <c r="F17" s="21"/>
       <c r="G17" s="4"/>
       <c r="H17" s="4"/>
     </row>
@@ -1129,14 +1133,16 @@
         <v>18</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="C19" s="17">
-        <v>33042</v>
+        <v>24116</v>
       </c>
       <c r="D19" s="17">
-        <v>36000</v>
-      </c>
+        <v>27000</v>
+      </c>
+      <c r="E19" s="15"/>
+      <c r="F19" s="21"/>
       <c r="G19" s="4"/>
       <c r="H19" s="4"/>
     </row>
@@ -1145,14 +1151,16 @@
         <v>19</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>17</v>
+        <v>39</v>
       </c>
       <c r="C20" s="17">
-        <v>20985</v>
+        <v>21080</v>
       </c>
       <c r="D20" s="17">
         <v>24000</v>
       </c>
+      <c r="E20" s="15"/>
+      <c r="F20" s="21"/>
       <c r="G20" s="4"/>
       <c r="H20" s="4"/>
     </row>
@@ -1161,15 +1169,15 @@
         <v>20</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="C21" s="17">
-        <v>14692</v>
+        <v>21039</v>
       </c>
       <c r="D21" s="17">
-        <v>18000</v>
-      </c>
-      <c r="E21" s="3"/>
+        <v>24000</v>
+      </c>
+      <c r="E21" s="15"/>
       <c r="F21" s="21"/>
       <c r="G21" s="4"/>
       <c r="H21" s="4"/>
@@ -1179,15 +1187,15 @@
         <v>21</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>26</v>
+        <v>43</v>
       </c>
       <c r="C22" s="17">
-        <v>14758</v>
+        <v>21020</v>
       </c>
       <c r="D22" s="17">
-        <v>18000</v>
-      </c>
-      <c r="E22" s="3"/>
+        <v>24000</v>
+      </c>
+      <c r="E22" s="15"/>
       <c r="F22" s="21"/>
       <c r="G22" s="4"/>
       <c r="H22" s="4"/>
@@ -1197,16 +1205,14 @@
         <v>22</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>27</v>
+        <v>12</v>
       </c>
       <c r="C23" s="17">
-        <v>29847</v>
+        <v>21012</v>
       </c>
       <c r="D23" s="17">
-        <v>33000</v>
-      </c>
-      <c r="E23" s="3"/>
-      <c r="F23" s="21"/>
+        <v>24000</v>
+      </c>
       <c r="G23" s="4"/>
       <c r="H23" s="4"/>
     </row>
@@ -1215,16 +1221,14 @@
         <v>23</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C24" s="17">
-        <v>32993</v>
+        <v>20985</v>
       </c>
       <c r="D24" s="17">
-        <v>36000</v>
-      </c>
-      <c r="E24" s="3"/>
-      <c r="F24" s="21"/>
+        <v>24000</v>
+      </c>
       <c r="G24" s="4"/>
       <c r="H24" s="4"/>
     </row>
@@ -1233,15 +1237,15 @@
         <v>24</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>15</v>
+        <v>49</v>
       </c>
       <c r="C25" s="17">
-        <v>29918</v>
+        <v>20929</v>
       </c>
       <c r="D25" s="17">
-        <v>33000</v>
-      </c>
-      <c r="E25" s="3"/>
+        <v>24000</v>
+      </c>
+      <c r="E25" s="15"/>
       <c r="F25" s="21"/>
       <c r="G25" s="4"/>
       <c r="H25" s="4"/>
@@ -1269,13 +1273,13 @@
         <v>26</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="C27" s="17">
-        <v>32945</v>
+        <v>18101</v>
       </c>
       <c r="D27" s="17">
-        <v>36000</v>
+        <v>21000</v>
       </c>
       <c r="E27" s="15"/>
       <c r="F27" s="21"/>
@@ -1287,13 +1291,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C28" s="17">
-        <v>14830</v>
+        <v>18033</v>
       </c>
       <c r="D28" s="17">
-        <v>18000</v>
+        <v>21000</v>
       </c>
       <c r="E28" s="15"/>
       <c r="F28" s="21"/>
@@ -1323,31 +1327,30 @@
         <v>29</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>35</v>
+        <v>11</v>
       </c>
       <c r="C30" s="17">
-        <v>21039</v>
+        <v>17822</v>
       </c>
       <c r="D30" s="17">
-        <v>24000</v>
-      </c>
-      <c r="E30" s="15"/>
-      <c r="F30" s="21"/>
+        <v>21000</v>
+      </c>
+      <c r="E30" s="3"/>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31" s="2">
         <v>30</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="C31" s="17">
-        <v>3024</v>
+        <v>14916</v>
       </c>
       <c r="D31" s="17">
-        <v>6000</v>
-      </c>
-      <c r="E31" s="15"/>
+        <v>18000</v>
+      </c>
+      <c r="E31" s="3"/>
       <c r="F31" s="21"/>
       <c r="G31" s="4"/>
       <c r="H31" s="4"/>
@@ -1357,16 +1360,14 @@
         <v>31</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>37</v>
+        <v>5</v>
       </c>
       <c r="C32" s="17">
-        <v>18033</v>
+        <v>14866</v>
       </c>
       <c r="D32" s="17">
-        <v>21000</v>
-      </c>
-      <c r="E32" s="15"/>
-      <c r="F32" s="21"/>
+        <v>18000</v>
+      </c>
       <c r="G32" s="4"/>
       <c r="H32" s="4"/>
     </row>
@@ -1375,13 +1376,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="C33" s="17">
-        <v>8986</v>
+        <v>14830</v>
       </c>
       <c r="D33" s="17">
-        <v>12000</v>
+        <v>18000</v>
       </c>
       <c r="E33" s="15"/>
       <c r="F33" s="21"/>
@@ -1393,13 +1394,13 @@
         <v>33</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
       <c r="C34" s="17">
-        <v>21080</v>
+        <v>14793</v>
       </c>
       <c r="D34" s="17">
-        <v>24000</v>
+        <v>18000</v>
       </c>
       <c r="E34" s="15"/>
       <c r="F34" s="21"/>
@@ -1411,15 +1412,15 @@
         <v>34</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="C35" s="17">
-        <v>8659</v>
+        <v>14758</v>
       </c>
       <c r="D35" s="17">
-        <v>12000</v>
-      </c>
-      <c r="E35" s="15"/>
+        <v>18000</v>
+      </c>
+      <c r="E35" s="3"/>
       <c r="F35" s="21"/>
       <c r="G35" s="4"/>
       <c r="H35" s="4"/>
@@ -1429,15 +1430,15 @@
         <v>35</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="C36" s="17">
-        <v>18101</v>
+        <v>14692</v>
       </c>
       <c r="D36" s="17">
-        <v>21000</v>
-      </c>
-      <c r="E36" s="15"/>
+        <v>18000</v>
+      </c>
+      <c r="E36" s="3"/>
       <c r="F36" s="21"/>
       <c r="G36" s="4"/>
       <c r="H36" s="4"/>
@@ -1465,13 +1466,13 @@
         <v>37</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C38" s="17">
-        <v>21020</v>
+        <v>14527</v>
       </c>
       <c r="D38" s="17">
-        <v>24000</v>
+        <v>18000</v>
       </c>
       <c r="E38" s="15"/>
       <c r="F38" s="21"/>
@@ -1501,16 +1502,15 @@
         <v>39</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>45</v>
+        <v>8</v>
       </c>
       <c r="C40" s="17">
-        <v>14793</v>
+        <v>12047</v>
       </c>
       <c r="D40" s="17">
-        <v>18000</v>
-      </c>
-      <c r="E40" s="15"/>
-      <c r="F40" s="21"/>
+        <v>15000</v>
+      </c>
+      <c r="E40" s="3"/>
       <c r="G40" s="4"/>
       <c r="H40" s="4"/>
     </row>
@@ -1519,10 +1519,10 @@
         <v>40</v>
       </c>
       <c r="B41" s="5" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="C41" s="17">
-        <v>8433</v>
+        <v>8986</v>
       </c>
       <c r="D41" s="17">
         <v>12000</v>
@@ -1537,13 +1537,13 @@
         <v>41</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C42" s="17">
-        <v>14527</v>
+        <v>8659</v>
       </c>
       <c r="D42" s="17">
-        <v>18000</v>
+        <v>12000</v>
       </c>
       <c r="E42" s="15"/>
       <c r="F42" s="21"/>
@@ -1555,13 +1555,13 @@
         <v>42</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="C43" s="17">
-        <v>24116</v>
+        <v>8433</v>
       </c>
       <c r="D43" s="17">
-        <v>27000</v>
+        <v>12000</v>
       </c>
       <c r="E43" s="15"/>
       <c r="F43" s="21"/>
@@ -1573,16 +1573,14 @@
         <v>43</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="C44" s="17">
-        <v>20929</v>
+        <v>6112</v>
       </c>
       <c r="D44" s="17">
-        <v>24000</v>
-      </c>
-      <c r="E44" s="15"/>
-      <c r="F44" s="21"/>
+        <v>9000</v>
+      </c>
       <c r="G44" s="4"/>
       <c r="H44" s="4"/>
     </row>
@@ -1591,13 +1589,13 @@
         <v>44</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>53</v>
+        <v>60</v>
       </c>
       <c r="C45" s="17">
-        <v>3136</v>
+        <v>6057</v>
       </c>
       <c r="D45" s="17">
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="G45" s="4"/>
       <c r="H45" s="4"/>
@@ -1607,13 +1605,13 @@
         <v>45</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="C46" s="17">
-        <v>2954</v>
+        <v>6025</v>
       </c>
       <c r="D46" s="17">
-        <v>6000</v>
+        <v>9000</v>
       </c>
       <c r="G46" s="4"/>
       <c r="H46" s="4"/>
@@ -1623,13 +1621,13 @@
         <v>46</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C47" s="17">
-        <v>6112</v>
+        <v>3136</v>
       </c>
       <c r="D47" s="17">
-        <v>9000</v>
+        <v>6000</v>
       </c>
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
@@ -1639,14 +1637,16 @@
         <v>47</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="C48" s="17">
-        <v>975</v>
+        <v>3024</v>
       </c>
       <c r="D48" s="17">
-        <v>3000</v>
-      </c>
+        <v>6000</v>
+      </c>
+      <c r="E48" s="15"/>
+      <c r="F48" s="21"/>
       <c r="G48" s="4"/>
       <c r="H48" s="4"/>
     </row>
@@ -1671,13 +1671,13 @@
         <v>49</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C50" s="17">
-        <v>6025</v>
+        <v>2954</v>
       </c>
       <c r="D50" s="17">
-        <v>9000</v>
+        <v>6000</v>
       </c>
       <c r="G50" s="4"/>
       <c r="H50" s="4"/>
@@ -1687,13 +1687,13 @@
         <v>50</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C51" s="17">
-        <v>6057</v>
+        <v>1005</v>
       </c>
       <c r="D51" s="17">
-        <v>9000</v>
+        <v>3000</v>
       </c>
       <c r="G51" s="4"/>
       <c r="H51" s="4"/>
@@ -1702,14 +1702,20 @@
       <c r="A52" s="2">
         <v>51</v>
       </c>
-      <c r="B52" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="C52" s="17">
-        <v>1005</v>
-      </c>
-      <c r="D52" s="17">
+      <c r="B52" s="23" t="s">
+        <v>59</v>
+      </c>
+      <c r="C52" s="24">
+        <v>982</v>
+      </c>
+      <c r="D52" s="24">
         <v>3000</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="F52" s="22" t="s">
+        <v>62</v>
       </c>
       <c r="G52" s="4"/>
       <c r="H52" s="4"/>
@@ -1718,20 +1724,14 @@
       <c r="A53" s="2">
         <v>52</v>
       </c>
-      <c r="B53" s="23" t="s">
-        <v>59</v>
-      </c>
-      <c r="C53" s="24">
-        <v>982</v>
-      </c>
-      <c r="D53" s="24">
+      <c r="B53" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C53" s="17">
+        <v>975</v>
+      </c>
+      <c r="D53" s="17">
         <v>3000</v>
-      </c>
-      <c r="E53" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="F53" s="22" t="s">
-        <v>62</v>
       </c>
       <c r="G53" s="4"/>
       <c r="H53" s="4"/>
@@ -1741,6 +1741,9 @@
     <row r="72" x14ac:dyDescent="0.35"/>
     <row r="73" x14ac:dyDescent="0.35"/>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B1:F73">
+    <sortCondition descending="1" ref="D1:D74"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>